<commit_message>
REFACTOR: dividir el estado REU-FEC-ASP en ronda 1 y ronda 2 (v11.0)
</commit_message>
<xml_diff>
--- a/Docs/Tabla de Estados - E3.xlsx
+++ b/Docs/Tabla de Estados - E3.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="65">
   <si>
     <t>Nro. Estado</t>
   </si>
@@ -122,7 +122,7 @@
     <t>Análisis pos reunión</t>
   </si>
   <si>
-    <t>Espacio previo a la aceptacion/rechazo de la inscripcion, en donde si hace falta, pueda re-subir documentos.</t>
+    <t>Espacio previo a la aceptacion/rechazo de la inscripcion, en donde si hace falta, el Academico puede actualizar la matriz de equivalencias y el horario de cursada.</t>
   </si>
   <si>
     <t>Aceptar analisis preliminar/equivalencias</t>
@@ -198,6 +198,15 @@
   </si>
   <si>
     <t>Inicio de E3</t>
+  </si>
+  <si>
+    <t>Reunión pendiente de fechas aspirante (1ª ronda)</t>
+  </si>
+  <si>
+    <t>Reunión pendiente de fechas aspirante (2ª ronda)</t>
+  </si>
+  <si>
+    <t>Reunión pendiente de fechas aspirante (1ª ronda o 2ª ronda)</t>
   </si>
 </sst>
 </file>
@@ -844,11 +853,11 @@
         <v>19</v>
       </c>
       <c r="F8" s="8" t="str">
-        <f t="shared" ref="F8:F11" si="2">G7</f>
+        <f t="shared" ref="F8:F10" si="2">G7</f>
         <v>Análisis preliminar pendiente</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>20</v>
+        <v>62</v>
       </c>
       <c r="H8" s="4" t="s">
         <v>21</v>
@@ -867,7 +876,7 @@
       </c>
       <c r="F9" s="8" t="str">
         <f t="shared" si="2"/>
-        <v>Reunión pendiente de fechas aspirante</v>
+        <v>Reunión pendiente de fechas aspirante (1ª ronda)</v>
       </c>
       <c r="G9" s="8" t="s">
         <v>23</v>
@@ -892,7 +901,7 @@
         <v>Reunión pendiente de fechas académico</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>20</v>
+        <v>63</v>
       </c>
       <c r="H10" s="4"/>
     </row>
@@ -907,9 +916,8 @@
       <c r="E11" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="F11" s="8" t="str">
-        <f t="shared" si="2"/>
-        <v>Reunión pendiente de fechas aspirante</v>
+      <c r="F11" s="8" t="s">
+        <v>64</v>
       </c>
       <c r="G11" s="8" t="s">
         <v>27</v>
@@ -938,7 +946,7 @@
       </c>
       <c r="F13" s="8" t="str">
         <f>G10</f>
-        <v>Reunión pendiente de fechas aspirante</v>
+        <v>Reunión pendiente de fechas aspirante (2ª ronda)</v>
       </c>
       <c r="G13" s="8" t="s">
         <v>30</v>

</xml_diff>

<commit_message>
ADDED: estado LEG-PEND y reprogramacion por no asistencia en la tabla de estados (v12.0)
</commit_message>
<xml_diff>
--- a/Docs/Tabla de Estados - E3.xlsx
+++ b/Docs/Tabla de Estados - E3.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="69">
   <si>
     <t>Nro. Estado</t>
   </si>
@@ -207,6 +207,18 @@
   </si>
   <si>
     <t>Reunión pendiente de fechas aspirante (1ª ronda o 2ª ronda)</t>
+  </si>
+  <si>
+    <t>Legalización pendiente</t>
+  </si>
+  <si>
+    <t>Indica que el aspirante no se presento</t>
+  </si>
+  <si>
+    <t>Indica que sus documentos NO estan legalizados</t>
+  </si>
+  <si>
+    <t>Avisa que ya legalizo sus documentos</t>
   </si>
 </sst>
 </file>
@@ -505,7 +517,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="C2:H47" displayName="ESTADOS" name="ESTADOS" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="C2:H50" displayName="ESTADOS" name="ESTADOS" id="1">
   <tableColumns count="6">
     <tableColumn name="Nro. Estado" id="1"/>
     <tableColumn name="Actor" id="2"/>
@@ -749,7 +761,7 @@
     </row>
     <row r="3" ht="22.5" customHeight="1">
       <c r="C3" s="2">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>6</v>
@@ -767,7 +779,7 @@
     </row>
     <row r="4" ht="22.5" customHeight="1">
       <c r="C4" s="5">
-        <f t="shared" ref="C4:C11" si="1">C3+1</f>
+        <f>C3+1</f>
         <v>2</v>
       </c>
       <c r="D4" s="2" t="s">
@@ -776,8 +788,9 @@
       <c r="E4" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F4" s="4" t="s">
-        <v>9</v>
+      <c r="F4" s="4" t="str">
+        <f>G3</f>
+        <v>Solicitud iniciada</v>
       </c>
       <c r="G4" s="4" t="s">
         <v>12</v>
@@ -786,7 +799,7 @@
     </row>
     <row r="5" ht="22.5" customHeight="1">
       <c r="C5" s="5">
-        <f t="shared" si="1"/>
+        <f>C4+1</f>
         <v>3</v>
       </c>
       <c r="D5" s="2" t="s">
@@ -795,8 +808,9 @@
       <c r="E5" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="F5" s="4" t="s">
-        <v>12</v>
+      <c r="F5" s="4" t="str">
+        <f>G4</f>
+        <v>Documentación pendiente de revisión</v>
       </c>
       <c r="G5" s="4" t="s">
         <v>15</v>
@@ -805,7 +819,7 @@
     </row>
     <row r="6" ht="22.5" customHeight="1">
       <c r="C6" s="5">
-        <f t="shared" si="1"/>
+        <f>C5+1</f>
         <v>4</v>
       </c>
       <c r="D6" s="2" t="s">
@@ -814,8 +828,9 @@
       <c r="E6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="F6" s="4" t="s">
-        <v>15</v>
+      <c r="F6" s="4" t="str">
+        <f>G5</f>
+        <v>Documentación rechazada</v>
       </c>
       <c r="G6" s="4" t="s">
         <v>12</v>
@@ -824,7 +839,7 @@
     </row>
     <row r="7" ht="22.5" customHeight="1">
       <c r="C7" s="5">
-        <f t="shared" si="1"/>
+        <f>C6+1</f>
         <v>5</v>
       </c>
       <c r="D7" s="2" t="s">
@@ -833,8 +848,9 @@
       <c r="E7" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F7" s="4" t="s">
-        <v>12</v>
+      <c r="F7" s="4" t="str">
+        <f>G6</f>
+        <v>Documentación pendiente de revisión</v>
       </c>
       <c r="G7" s="4" t="s">
         <v>18</v>
@@ -843,7 +859,7 @@
     </row>
     <row r="8" ht="22.5" customHeight="1">
       <c r="C8" s="6">
-        <f t="shared" si="1"/>
+        <f>C7+1</f>
         <v>6</v>
       </c>
       <c r="D8" s="7" t="s">
@@ -853,7 +869,7 @@
         <v>19</v>
       </c>
       <c r="F8" s="8" t="str">
-        <f t="shared" ref="F8:F10" si="2">G7</f>
+        <f>G7</f>
         <v>Análisis preliminar pendiente</v>
       </c>
       <c r="G8" s="8" t="s">
@@ -865,7 +881,7 @@
     </row>
     <row r="9" ht="22.5" customHeight="1">
       <c r="C9" s="6">
-        <f t="shared" si="1"/>
+        <f>C8+1</f>
         <v>7</v>
       </c>
       <c r="D9" s="7" t="s">
@@ -875,7 +891,7 @@
         <v>22</v>
       </c>
       <c r="F9" s="8" t="str">
-        <f t="shared" si="2"/>
+        <f>G8</f>
         <v>Reunión pendiente de fechas aspirante (1ª ronda)</v>
       </c>
       <c r="G9" s="8" t="s">
@@ -887,7 +903,7 @@
     </row>
     <row r="10" ht="22.5" customHeight="1">
       <c r="C10" s="6">
-        <f t="shared" si="1"/>
+        <f>C9+1</f>
         <v>8</v>
       </c>
       <c r="D10" s="7" t="s">
@@ -897,7 +913,7 @@
         <v>25</v>
       </c>
       <c r="F10" s="8" t="str">
-        <f t="shared" si="2"/>
+        <f>G9</f>
         <v>Reunión pendiente de fechas académico</v>
       </c>
       <c r="G10" s="8" t="s">
@@ -907,7 +923,7 @@
     </row>
     <row r="11" ht="22.5" customHeight="1">
       <c r="C11" s="6">
-        <f t="shared" si="1"/>
+        <f>C10+1</f>
         <v>9</v>
       </c>
       <c r="D11" s="7" t="s">
@@ -936,7 +952,7 @@
     </row>
     <row r="13" ht="22.5" customHeight="1">
       <c r="C13" s="7">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="D13" s="7" t="s">
         <v>6</v>
@@ -944,9 +960,8 @@
       <c r="E13" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="F13" s="8" t="str">
-        <f>G10</f>
-        <v>Reunión pendiente de fechas aspirante (2ª ronda)</v>
+      <c r="F13" s="8" t="s">
+        <v>63</v>
       </c>
       <c r="G13" s="8" t="s">
         <v>30</v>
@@ -987,294 +1002,332 @@
     </row>
     <row r="16" ht="22.5" customHeight="1">
       <c r="C16" s="7">
-        <v>12.0</v>
+        <v>12</v>
       </c>
       <c r="D16" s="7" t="s">
         <v>13</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>34</v>
+        <v>66</v>
       </c>
       <c r="F16" s="8" t="str">
         <f>G14</f>
         <v>Reunión pendiente de realización</v>
       </c>
       <c r="G16" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="H16" s="4" t="s">
-        <v>36</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="H16" s="4"/>
     </row>
     <row r="17" ht="22.5" customHeight="1">
       <c r="C17" s="7">
-        <f t="shared" ref="C17:C18" si="3">C16+1</f>
+        <f>C16+1</f>
         <v>13</v>
       </c>
       <c r="D17" s="7" t="s">
         <v>13</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="F17" s="8" t="str">
-        <f>G16</f>
-        <v>Análisis pos reunión</v>
+        <v>34</v>
+      </c>
+      <c r="F17" s="8" t="s">
+        <v>27</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="H17" s="4"/>
+        <v>35</v>
+      </c>
+      <c r="H17" s="4" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="18" ht="22.5" customHeight="1">
       <c r="C18" s="7">
-        <f t="shared" si="3"/>
+        <f>C17+1</f>
         <v>14</v>
       </c>
       <c r="D18" s="7" t="s">
         <v>13</v>
       </c>
       <c r="E18" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="F18" s="8" t="str">
+        <f>G17</f>
+        <v>Análisis pos reunión</v>
+      </c>
+      <c r="G18" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="H18" s="4"/>
+    </row>
+    <row r="19" ht="22.5" customHeight="1">
+      <c r="C19" s="7">
+        <f>C18+1</f>
+        <v>15</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E19" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="F18" s="8" t="s">
+      <c r="F19" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="G18" s="8" t="s">
+      <c r="G19" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="H18" s="4" t="s">
+      <c r="H19" s="4" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="19" ht="22.5" customHeight="1">
-      <c r="C19" s="9"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="9"/>
-      <c r="F19" s="9"/>
-      <c r="G19" s="9"/>
-      <c r="H19" s="9"/>
-    </row>
-    <row r="20" ht="22.5" customHeight="1">
-      <c r="C20" s="7">
-        <v>15.0</v>
-      </c>
-      <c r="D20" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="E20" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="F20" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="G20" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="H20" s="4" t="s">
-        <v>44</v>
-      </c>
+    <row r="20" ht="24.0" customHeight="1">
+      <c r="C20" s="9"/>
+      <c r="D20" s="9"/>
+      <c r="E20" s="9"/>
+      <c r="F20" s="9"/>
+      <c r="G20" s="9"/>
+      <c r="H20" s="9"/>
     </row>
     <row r="21" ht="22.5" customHeight="1">
       <c r="C21" s="7">
-        <f t="shared" ref="C21:C23" si="4">C20+1</f>
         <v>16</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="E21" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="F21" s="11" t="str">
-        <f t="shared" ref="F21:F23" si="5">G20</f>
-        <v>Análisis de documentos legalizados</v>
+        <v>42</v>
+      </c>
+      <c r="F21" s="11" t="s">
+        <v>38</v>
       </c>
       <c r="G21" s="11" t="s">
-        <v>46</v>
-      </c>
-      <c r="H21" s="4"/>
+        <v>43</v>
+      </c>
+      <c r="H21" s="4" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="22" ht="22.5" customHeight="1">
       <c r="C22" s="7">
-        <f t="shared" si="4"/>
+        <f>C21+1</f>
         <v>17</v>
       </c>
       <c r="D22" s="10" t="s">
         <v>6</v>
       </c>
       <c r="E22" s="11" t="s">
-        <v>47</v>
-      </c>
-      <c r="F22" s="11" t="str">
-        <f t="shared" si="5"/>
-        <v>Documentos legalizados rechazados</v>
+        <v>67</v>
+      </c>
+      <c r="F22" s="11" t="s">
+        <v>38</v>
       </c>
       <c r="G22" s="11" t="s">
-        <v>43</v>
+        <v>65</v>
       </c>
       <c r="H22" s="4"/>
     </row>
     <row r="23" ht="22.5" customHeight="1">
       <c r="C23" s="7">
-        <f t="shared" si="4"/>
+        <f>C22+1</f>
         <v>18</v>
       </c>
       <c r="D23" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="E23" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="F23" s="12" t="str">
+        <f>G22</f>
+        <v>Legalización pendiente</v>
+      </c>
+      <c r="G23" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="H23" s="4"/>
+    </row>
+    <row r="24" ht="22.5" customHeight="1">
+      <c r="C24" s="7">
+        <f>C23+1</f>
+        <v>19</v>
+      </c>
+      <c r="D24" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="E23" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="F23" s="12" t="str">
-        <f t="shared" si="5"/>
+      <c r="E24" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="F24" s="11" t="str">
+        <f>G23</f>
         <v>Análisis de documentos legalizados</v>
       </c>
-      <c r="G23" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="H23" s="4" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="24" ht="22.5" customHeight="1">
-      <c r="C24" s="9"/>
-      <c r="D24" s="9"/>
-      <c r="E24" s="9"/>
-      <c r="F24" s="9"/>
-      <c r="G24" s="9"/>
-      <c r="H24" s="9"/>
+      <c r="G24" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="H24" s="4"/>
     </row>
     <row r="25" ht="22.5" customHeight="1">
       <c r="C25" s="7">
-        <v>19.0</v>
-      </c>
-      <c r="D25" s="13" t="s">
-        <v>51</v>
+        <f>C24+1</f>
+        <v>20</v>
+      </c>
+      <c r="D25" s="10" t="s">
+        <v>6</v>
       </c>
       <c r="E25" s="11" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="F25" s="11" t="str">
-        <f>G23</f>
-        <v>Solicitud de cupón de pago</v>
+        <f>G24</f>
+        <v>Documentos legalizados rechazados</v>
       </c>
       <c r="G25" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="H25" s="14"/>
+        <v>43</v>
+      </c>
+      <c r="H25" s="4"/>
     </row>
     <row r="26" ht="22.5" customHeight="1">
       <c r="C26" s="7">
-        <v>20.0</v>
-      </c>
-      <c r="D26" s="13" t="s">
-        <v>6</v>
+        <f>C25+1</f>
+        <v>21</v>
+      </c>
+      <c r="D26" s="10" t="s">
+        <v>13</v>
       </c>
       <c r="E26" s="11" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="F26" s="11" t="str">
         <f>G25</f>
+        <v>Análisis de documentos legalizados</v>
+      </c>
+      <c r="G26" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="H26" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="27" ht="24.0" customHeight="1">
+      <c r="C27" s="9"/>
+      <c r="D27" s="9"/>
+      <c r="E27" s="9"/>
+      <c r="F27" s="9"/>
+      <c r="G27" s="9"/>
+      <c r="H27" s="9"/>
+    </row>
+    <row r="28" ht="22.5" customHeight="1">
+      <c r="C28" s="7">
+        <v>22</v>
+      </c>
+      <c r="D28" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="E28" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="F28" s="11" t="str">
+        <f>G26</f>
+        <v>Solicitud de cupón de pago</v>
+      </c>
+      <c r="G28" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="H28" s="14"/>
+    </row>
+    <row r="29" ht="22.5" customHeight="1">
+      <c r="C29" s="7">
+        <f>C28+1</f>
+        <v>23</v>
+      </c>
+      <c r="D29" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="E29" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="F29" s="11" t="str">
+        <f>G28</f>
         <v>Pago de cupón por aspirante</v>
       </c>
-      <c r="G26" s="11" t="s">
+      <c r="G29" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="H26" s="11" t="s">
+      <c r="H29" s="11" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="27" ht="22.5" customHeight="1">
-      <c r="C27" s="2">
-        <v>21</v>
-      </c>
-      <c r="D27" s="13" t="s">
+    <row r="30" ht="22.5" customHeight="1">
+      <c r="C30" s="2">
+        <f>C29+1</f>
+        <v>24</v>
+      </c>
+      <c r="D30" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="E27" s="11" t="s">
+      <c r="E30" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="F27" s="4" t="str">
-        <f>G26</f>
+      <c r="F30" s="4" t="str">
+        <f>G29</f>
         <v>Control de pago</v>
       </c>
-      <c r="G27" s="11" t="s">
+      <c r="G30" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="H27" s="11"/>
-    </row>
-    <row r="28" ht="22.5" customHeight="1">
-      <c r="C28" s="2">
-        <v>22</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="H30" s="11"/>
+    </row>
+    <row r="31" ht="22.5" customHeight="1">
+      <c r="C31" s="2">
+        <f>C30+1</f>
+        <v>25</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t>Reenvía comprobante</t>
         </is>
       </c>
-      <c r="F28" s="2" t="str">
-        <f t="shared" ref="F28:F29" si="6">G27</f>
+      <c r="F31" s="2" t="str">
+        <f>G30</f>
         <v>Reenvío de comprobante</v>
       </c>
-      <c r="G28" s="11" t="s">
+      <c r="G31" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="H28" s="11"/>
-    </row>
-    <row r="29" ht="22.5" customHeight="1">
-      <c r="C29" s="2">
-        <v>23</v>
-      </c>
-      <c r="D29" s="13" t="s">
+      <c r="H31" s="11"/>
+    </row>
+    <row r="32" ht="22.5" customHeight="1">
+      <c r="C32" s="2">
+        <f>C31+1</f>
+        <v>26</v>
+      </c>
+      <c r="D32" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="E29" s="11" t="s">
+      <c r="E32" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="F29" s="4" t="str">
-        <f t="shared" si="6"/>
+      <c r="F32" s="4" t="str">
+        <f>G31</f>
         <v>Control de pago</v>
       </c>
-      <c r="G29" s="11" t="s">
+      <c r="G32" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="H29" s="11"/>
-    </row>
-    <row r="30" ht="22.5" customHeight="1">
-      <c r="C30" s="9"/>
-      <c r="D30" s="9"/>
-      <c r="E30" s="9"/>
-      <c r="F30" s="9"/>
-      <c r="G30" s="9"/>
-      <c r="H30" s="9"/>
-    </row>
-    <row r="31" ht="22.5" customHeight="1">
-      <c r="C31" s="7"/>
-      <c r="D31" s="13"/>
-      <c r="E31" s="11"/>
-      <c r="F31" s="12"/>
-      <c r="G31" s="12"/>
-      <c r="H31" s="11"/>
-    </row>
-    <row r="32" ht="22.5" customHeight="1">
-      <c r="C32" s="7"/>
-      <c r="D32" s="13"/>
-      <c r="E32" s="11"/>
-      <c r="F32" s="12"/>
-      <c r="G32" s="12"/>
       <c r="H32" s="11"/>
     </row>
-    <row r="33" ht="22.5" customHeight="1">
-      <c r="C33" s="5"/>
-      <c r="D33" s="13"/>
-      <c r="E33" s="11"/>
-      <c r="F33" s="12"/>
-      <c r="G33" s="12"/>
-      <c r="H33" s="11"/>
+    <row r="33" ht="24.0" customHeight="1">
+      <c r="C33" s="9"/>
+      <c r="D33" s="9"/>
+      <c r="E33" s="9"/>
+      <c r="F33" s="9"/>
+      <c r="G33" s="9"/>
+      <c r="H33" s="9"/>
     </row>
     <row r="34" ht="22.5" customHeight="1">
       <c r="C34" s="7"/>
@@ -1285,108 +1338,132 @@
       <c r="H34" s="11"/>
     </row>
     <row r="35" ht="22.5" customHeight="1">
-      <c r="C35" s="15"/>
-      <c r="D35" s="16"/>
-      <c r="E35" s="17"/>
-      <c r="F35" s="17"/>
-      <c r="G35" s="17"/>
-      <c r="H35" s="18"/>
+      <c r="C35" s="7"/>
+      <c r="D35" s="13"/>
+      <c r="E35" s="11"/>
+      <c r="F35" s="12"/>
+      <c r="G35" s="12"/>
+      <c r="H35" s="11"/>
     </row>
     <row r="36" ht="22.5" customHeight="1">
-      <c r="C36" s="19"/>
-      <c r="D36" s="20"/>
-      <c r="E36" s="21"/>
-      <c r="F36" s="21"/>
-      <c r="G36" s="21"/>
-      <c r="H36" s="22"/>
+      <c r="C36" s="5"/>
+      <c r="D36" s="13"/>
+      <c r="E36" s="11"/>
+      <c r="F36" s="12"/>
+      <c r="G36" s="12"/>
+      <c r="H36" s="11"/>
     </row>
     <row r="37" ht="22.5" customHeight="1">
-      <c r="C37" s="15"/>
-      <c r="D37" s="16"/>
-      <c r="E37" s="17"/>
-      <c r="F37" s="17"/>
-      <c r="G37" s="17"/>
-      <c r="H37" s="18"/>
+      <c r="C37" s="7"/>
+      <c r="D37" s="13"/>
+      <c r="E37" s="11"/>
+      <c r="F37" s="12"/>
+      <c r="G37" s="12"/>
+      <c r="H37" s="11"/>
     </row>
     <row r="38" ht="22.5" customHeight="1">
-      <c r="C38" s="19"/>
-      <c r="D38" s="20"/>
-      <c r="E38" s="21"/>
-      <c r="F38" s="21"/>
-      <c r="G38" s="21"/>
-      <c r="H38" s="22"/>
+      <c r="C38" s="15"/>
+      <c r="D38" s="16"/>
+      <c r="E38" s="17"/>
+      <c r="F38" s="17"/>
+      <c r="G38" s="17"/>
+      <c r="H38" s="18"/>
     </row>
     <row r="39" ht="22.5" customHeight="1">
-      <c r="C39" s="15"/>
-      <c r="D39" s="16"/>
-      <c r="E39" s="17"/>
-      <c r="F39" s="17"/>
-      <c r="G39" s="17"/>
-      <c r="H39" s="18"/>
+      <c r="C39" s="19"/>
+      <c r="D39" s="20"/>
+      <c r="E39" s="21"/>
+      <c r="F39" s="21"/>
+      <c r="G39" s="21"/>
+      <c r="H39" s="22"/>
     </row>
     <row r="40" ht="22.5" customHeight="1">
-      <c r="C40" s="19"/>
-      <c r="D40" s="20"/>
-      <c r="E40" s="21"/>
-      <c r="F40" s="21"/>
-      <c r="G40" s="21"/>
-      <c r="H40" s="22"/>
+      <c r="C40" s="15"/>
+      <c r="D40" s="16"/>
+      <c r="E40" s="17"/>
+      <c r="F40" s="17"/>
+      <c r="G40" s="17"/>
+      <c r="H40" s="18"/>
     </row>
     <row r="41" ht="22.5" customHeight="1">
-      <c r="C41" s="15"/>
-      <c r="D41" s="16"/>
-      <c r="E41" s="17"/>
-      <c r="F41" s="17"/>
-      <c r="G41" s="17"/>
-      <c r="H41" s="18"/>
+      <c r="C41" s="19"/>
+      <c r="D41" s="20"/>
+      <c r="E41" s="21"/>
+      <c r="F41" s="21"/>
+      <c r="G41" s="21"/>
+      <c r="H41" s="22"/>
     </row>
     <row r="42" ht="22.5" customHeight="1">
-      <c r="C42" s="19"/>
-      <c r="D42" s="20"/>
-      <c r="E42" s="21"/>
-      <c r="F42" s="21"/>
-      <c r="G42" s="21"/>
-      <c r="H42" s="22"/>
+      <c r="C42" s="15"/>
+      <c r="D42" s="16"/>
+      <c r="E42" s="17"/>
+      <c r="F42" s="17"/>
+      <c r="G42" s="17"/>
+      <c r="H42" s="18"/>
     </row>
     <row r="43" ht="22.5" customHeight="1">
-      <c r="C43" s="15"/>
-      <c r="D43" s="16"/>
-      <c r="E43" s="17"/>
-      <c r="F43" s="17"/>
-      <c r="G43" s="17"/>
-      <c r="H43" s="18"/>
+      <c r="C43" s="19"/>
+      <c r="D43" s="20"/>
+      <c r="E43" s="21"/>
+      <c r="F43" s="21"/>
+      <c r="G43" s="21"/>
+      <c r="H43" s="22"/>
     </row>
     <row r="44" ht="22.5" customHeight="1">
-      <c r="C44" s="19"/>
-      <c r="D44" s="20"/>
-      <c r="E44" s="21"/>
-      <c r="F44" s="21"/>
-      <c r="G44" s="21"/>
-      <c r="H44" s="22"/>
+      <c r="C44" s="15"/>
+      <c r="D44" s="16"/>
+      <c r="E44" s="17"/>
+      <c r="F44" s="17"/>
+      <c r="G44" s="17"/>
+      <c r="H44" s="18"/>
     </row>
     <row r="45" ht="22.5" customHeight="1">
-      <c r="C45" s="15"/>
-      <c r="D45" s="16"/>
-      <c r="E45" s="17"/>
-      <c r="F45" s="17"/>
-      <c r="G45" s="17"/>
-      <c r="H45" s="18"/>
+      <c r="C45" s="19"/>
+      <c r="D45" s="20"/>
+      <c r="E45" s="21"/>
+      <c r="F45" s="21"/>
+      <c r="G45" s="21"/>
+      <c r="H45" s="22"/>
     </row>
     <row r="46" ht="22.5" customHeight="1">
-      <c r="C46" s="19"/>
-      <c r="D46" s="20"/>
-      <c r="E46" s="21"/>
-      <c r="F46" s="21"/>
-      <c r="G46" s="21"/>
-      <c r="H46" s="22"/>
+      <c r="C46" s="15"/>
+      <c r="D46" s="16"/>
+      <c r="E46" s="17"/>
+      <c r="F46" s="17"/>
+      <c r="G46" s="17"/>
+      <c r="H46" s="18"/>
     </row>
     <row r="47" ht="22.5" customHeight="1">
-      <c r="C47" s="15"/>
-      <c r="D47" s="16"/>
-      <c r="E47" s="17"/>
-      <c r="F47" s="17"/>
-      <c r="G47" s="17"/>
-      <c r="H47" s="18"/>
+      <c r="C47" s="19"/>
+      <c r="D47" s="20"/>
+      <c r="E47" s="21"/>
+      <c r="F47" s="21"/>
+      <c r="G47" s="21"/>
+      <c r="H47" s="22"/>
+    </row>
+    <row r="48" ht="22.5" customHeight="1">
+      <c r="C48" s="15"/>
+      <c r="D48" s="16"/>
+      <c r="E48" s="17"/>
+      <c r="F48" s="17"/>
+      <c r="G48" s="17"/>
+      <c r="H48" s="18"/>
+    </row>
+    <row r="49" ht="22.5" customHeight="1">
+      <c r="C49" s="19"/>
+      <c r="D49" s="20"/>
+      <c r="E49" s="21"/>
+      <c r="F49" s="21"/>
+      <c r="G49" s="21"/>
+      <c r="H49" s="22"/>
+    </row>
+    <row r="50" ht="22.5" customHeight="1">
+      <c r="C50" s="15"/>
+      <c r="D50" s="16"/>
+      <c r="E50" s="17"/>
+      <c r="F50" s="17"/>
+      <c r="G50" s="17"/>
+      <c r="H50" s="18"/>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>

</xml_diff>